<commit_message>
Update Actions.txt to change notifyEmail to a specific address and refine contract type validation logic. Enhance frida-core.mdc and frida-web.mdc with guidelines on the use of system notifications, emphasizing their exceptional nature and restrictions in web automation. Update binary Excel files for consistency.
</commit_message>
<xml_diff>
--- a/Inputs/COMPRA PERGAMINO ESPECIAL - 100126.xlsx
+++ b/Inputs/COMPRA PERGAMINO ESPECIAL - 100126.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rodrigo.gracia\Documents\Projects\ECOM\Inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{795F4CE6-EAA6-4ACB-B47F-466C2226434D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72AAB96A-56D9-4B30-B431-804FF9839BFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-3210" yWindow="7570" windowWidth="19420" windowHeight="11500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="114">
   <si>
     <t>ContractType</t>
   </si>
@@ -884,6 +884,12 @@
   </si>
   <si>
     <t>SAPBot_2026-03-02_16-43-28</t>
+  </si>
+  <si>
+    <t>Processing</t>
+  </si>
+  <si>
+    <t>SAPBot_2026-03-03_12-20-35</t>
   </si>
 </sst>
 </file>
@@ -1495,50 +1501,50 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AW13"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.1796875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="15.140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="19" style="1" customWidth="1"/>
     <col min="3" max="3" width="13" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="12.453125" style="13" customWidth="1"/>
-    <col min="6" max="6" width="6.7265625" customWidth="1"/>
-    <col min="7" max="7" width="9.453125" customWidth="1"/>
-    <col min="8" max="8" width="9.81640625" style="11" customWidth="1"/>
-    <col min="9" max="10" width="16.81640625" style="13" customWidth="1"/>
-    <col min="11" max="11" width="11.81640625" customWidth="1"/>
-    <col min="12" max="12" width="19.81640625" customWidth="1"/>
-    <col min="13" max="13" width="33.81640625" customWidth="1"/>
-    <col min="14" max="14" width="10.7265625" customWidth="1"/>
-    <col min="15" max="15" width="20.26953125" customWidth="1"/>
-    <col min="16" max="16" width="26.26953125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.81640625" customWidth="1"/>
-    <col min="18" max="19" width="15.54296875" customWidth="1"/>
-    <col min="20" max="21" width="18.7265625" customWidth="1"/>
-    <col min="22" max="22" width="18.7265625" style="13" customWidth="1"/>
-    <col min="23" max="24" width="18.7265625" customWidth="1"/>
-    <col min="25" max="25" width="23.453125" customWidth="1"/>
-    <col min="26" max="27" width="18.7265625" customWidth="1"/>
-    <col min="28" max="28" width="17.54296875" customWidth="1"/>
-    <col min="29" max="29" width="12.26953125" customWidth="1"/>
-    <col min="30" max="30" width="21.1796875" customWidth="1"/>
-    <col min="31" max="31" width="12.26953125" style="11" customWidth="1"/>
-    <col min="32" max="32" width="12.26953125" customWidth="1"/>
+    <col min="5" max="5" width="12.42578125" style="13" customWidth="1"/>
+    <col min="6" max="6" width="6.7109375" customWidth="1"/>
+    <col min="7" max="7" width="9.42578125" customWidth="1"/>
+    <col min="8" max="8" width="9.85546875" style="11" customWidth="1"/>
+    <col min="9" max="10" width="16.85546875" style="13" customWidth="1"/>
+    <col min="11" max="11" width="11.85546875" customWidth="1"/>
+    <col min="12" max="12" width="19.85546875" customWidth="1"/>
+    <col min="13" max="13" width="33.85546875" customWidth="1"/>
+    <col min="14" max="14" width="10.7109375" customWidth="1"/>
+    <col min="15" max="15" width="20.28515625" customWidth="1"/>
+    <col min="16" max="16" width="26.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.85546875" customWidth="1"/>
+    <col min="18" max="19" width="15.5703125" customWidth="1"/>
+    <col min="20" max="21" width="18.7109375" customWidth="1"/>
+    <col min="22" max="22" width="18.7109375" style="13" customWidth="1"/>
+    <col min="23" max="24" width="18.7109375" customWidth="1"/>
+    <col min="25" max="25" width="23.42578125" customWidth="1"/>
+    <col min="26" max="27" width="18.7109375" customWidth="1"/>
+    <col min="28" max="28" width="17.5703125" customWidth="1"/>
+    <col min="29" max="29" width="12.28515625" customWidth="1"/>
+    <col min="30" max="30" width="21.140625" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="11" customWidth="1"/>
+    <col min="32" max="32" width="12.28515625" customWidth="1"/>
     <col min="33" max="33" width="14" customWidth="1"/>
-    <col min="34" max="36" width="10.7265625" customWidth="1"/>
-    <col min="37" max="37" width="18.453125" customWidth="1"/>
-    <col min="38" max="38" width="32.453125" customWidth="1"/>
-    <col min="39" max="39" width="23.1796875" customWidth="1"/>
-    <col min="40" max="40" width="28.1796875" customWidth="1"/>
-    <col min="41" max="41" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="42" max="44" width="28.54296875" customWidth="1"/>
-    <col min="45" max="45" width="22.81640625" customWidth="1"/>
-    <col min="46" max="46" width="20.1796875" customWidth="1"/>
-    <col min="47" max="47" width="28.54296875" customWidth="1"/>
+    <col min="34" max="36" width="10.7109375" customWidth="1"/>
+    <col min="37" max="37" width="18.42578125" customWidth="1"/>
+    <col min="38" max="38" width="32.42578125" customWidth="1"/>
+    <col min="39" max="39" width="23.140625" customWidth="1"/>
+    <col min="40" max="40" width="28.140625" customWidth="1"/>
+    <col min="41" max="41" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="42" max="44" width="28.5703125" customWidth="1"/>
+    <col min="45" max="45" width="22.85546875" customWidth="1"/>
+    <col min="46" max="46" width="20.140625" customWidth="1"/>
+    <col min="47" max="47" width="28.5703125" customWidth="1"/>
     <col min="49" max="49" width="56" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:49" ht="37.4" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:49" ht="37.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1687,7 +1693,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="2" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
         <v>46</v>
       </c>
@@ -1802,7 +1808,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="3" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
         <v>46</v>
       </c>
@@ -1915,7 +1921,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
         <v>46</v>
       </c>
@@ -2028,7 +2034,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="5" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
         <v>46</v>
       </c>
@@ -2143,10 +2149,10 @@
         <v>107</v>
       </c>
       <c r="AW5" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="6" spans="1:49" x14ac:dyDescent="0.35">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="6" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
         <v>46</v>
       </c>
@@ -2259,13 +2265,13 @@
         <v>55</v>
       </c>
       <c r="AV6" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="AW6" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="7" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
         <v>46</v>
       </c>
@@ -2382,7 +2388,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="8" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A8" s="15" t="s">
         <v>46</v>
       </c>
@@ -2500,19 +2506,19 @@
         <v>110</v>
       </c>
     </row>
-    <row r="11" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A11" s="8"/>
       <c r="B11" s="1" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="12" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A12" s="9"/>
       <c r="B12" s="1" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="13" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A13" s="10"/>
       <c r="B13" s="1" t="s">
         <v>91</v>
@@ -2528,23 +2534,23 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:L21"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:L22"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.1796875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10.81640625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="15.140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="10.85546875" style="1" customWidth="1"/>
     <col min="3" max="3" width="13" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="6.7265625" customWidth="1"/>
-    <col min="6" max="6" width="9.453125" customWidth="1"/>
-    <col min="7" max="7" width="9.81640625" customWidth="1"/>
-    <col min="8" max="9" width="16.81640625" customWidth="1"/>
-    <col min="10" max="10" width="11.81640625" customWidth="1"/>
-    <col min="11" max="11" width="33.81640625" customWidth="1"/>
-    <col min="12" max="12" width="10.7265625" customWidth="1"/>
+    <col min="5" max="5" width="6.7109375" customWidth="1"/>
+    <col min="6" max="6" width="9.42578125" customWidth="1"/>
+    <col min="7" max="7" width="9.85546875" customWidth="1"/>
+    <col min="8" max="9" width="16.85546875" customWidth="1"/>
+    <col min="10" max="10" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="33.85546875" customWidth="1"/>
+    <col min="12" max="12" width="10.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="27" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2582,7 +2588,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>2</v>
       </c>
@@ -2599,7 +2605,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>3</v>
       </c>
@@ -2616,7 +2622,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -2633,7 +2639,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>3</v>
       </c>
@@ -2650,7 +2656,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>4</v>
       </c>
@@ -2667,7 +2673,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>5</v>
       </c>
@@ -2684,7 +2690,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>6</v>
       </c>
@@ -2701,7 +2707,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>7</v>
       </c>
@@ -2718,7 +2724,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>8</v>
       </c>
@@ -2735,7 +2741,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>2</v>
       </c>
@@ -2752,7 +2758,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>3</v>
       </c>
@@ -2769,7 +2775,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>4</v>
       </c>
@@ -2786,7 +2792,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>5</v>
       </c>
@@ -2803,7 +2809,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>6</v>
       </c>
@@ -2820,7 +2826,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>7</v>
       </c>
@@ -2837,7 +2843,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>8</v>
       </c>
@@ -2854,7 +2860,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>5</v>
       </c>
@@ -2871,7 +2877,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>6</v>
       </c>
@@ -2884,8 +2890,11 @@
       <c r="D19" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E19" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>7</v>
       </c>
@@ -2899,7 +2908,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>8</v>
       </c>
@@ -2911,6 +2920,20 @@
       </c>
       <c r="D21" t="s">
         <v>111</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="1">
+        <v>5</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C22" s="25">
+        <v>46084.514606481483</v>
+      </c>
+      <c r="D22" t="s">
+        <v>113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>